<commit_message>
site build 2026-10-08 19:28
</commit_message>
<xml_diff>
--- a/models/sovereigns/Angola_Sovereign_Model.xlsx
+++ b/models/sovereigns/Angola_Sovereign_Model.xlsx
@@ -816,16 +816,34 @@
           <t>fiscal_balance_pct_gdp</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n"/>
+      <c r="B10" s="2" t="n">
+        <v>-2.4</v>
+      </c>
       <c r="C10" t="inlineStr">
         <is>
           <t>% GDP</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026E</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>IMF WEO</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>08-Oct-26</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -915,16 +933,34 @@
           <t>fdi_net_pct_gdp</t>
         </is>
       </c>
-      <c r="B15" s="2" t="n"/>
+      <c r="B15" s="2" t="n">
+        <v>1.814</v>
+      </c>
       <c r="C15" t="inlineStr">
         <is>
           <t>% GDP</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>World Bank WDI</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>08-Oct-26</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1066,16 +1102,34 @@
           <t>nominal_gdp_usd_bn</t>
         </is>
       </c>
-      <c r="B22" s="2" t="n"/>
+      <c r="B22" s="2" t="n">
+        <v>152.354</v>
+      </c>
       <c r="C22" t="inlineStr">
         <is>
           <t>USD bn</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>2026E</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>IMF WEO</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>08-Oct-26</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">

</xml_diff>

<commit_message>
site build 2026-10-08 21:36
</commit_message>
<xml_diff>
--- a/models/sovereigns/Angola_Sovereign_Model.xlsx
+++ b/models/sovereigns/Angola_Sovereign_Model.xlsx
@@ -700,12 +700,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>INE, IPCN Aug-26</t>
+          <t>INE</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>30-Aug-26</t>
+          <t>08-Oct-26</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -731,12 +731,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>IMF, 2026 Article IV Consultation</t>
+          <t>IMF</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>01-May-26</t>
+          <t>08-Oct-26</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -779,17 +779,17 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>MINFIN / IMF</t>
+          <t>MINFIN/IMF</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>01-May-26</t>
+          <t>08-Oct-26</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Public debt, end-2025; statutory ceiling 60% under Fiscal Sustainability Law</t>
+          <t>public debt, approx., end-2025</t>
         </is>
       </c>
     </row>
@@ -839,11 +839,7 @@
           <t>08-Oct-26</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -917,12 +913,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>IMF / BNA</t>
+          <t>IMF/BNA</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>01-May-26</t>
+          <t>08-Oct-26</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -956,11 +952,7 @@
           <t>08-Oct-26</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -969,7 +961,7 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>14.9</v>
+        <v>15.821</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -978,22 +970,22 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Q2-26</t>
+          <t>Aug-26</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>IMF International Liquidity</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>30-Jun-26</t>
+          <t>08-Oct-26</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>BNA gross international reserves</t>
+          <t>gross incl. gold ($13.192B ex gold plus $2.629B gold)</t>
         </is>
       </c>
     </row>
@@ -1003,16 +995,34 @@
           <t>net_reserves_usd_bn</t>
         </is>
       </c>
-      <c r="B17" s="2" t="n"/>
+      <c r="B17" s="2" t="n">
+        <v>0.618</v>
+      </c>
       <c r="C17" t="inlineStr">
         <is>
           <t>USD bn</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>IMF reserve template</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>08-Oct-26</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>official reserve assets net of one-year predetermined and contingent drains (IMF reserve template)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1040,7 +1050,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>30-Jun-26</t>
+          <t>08-Oct-26</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
@@ -1103,7 +1113,7 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>152.354</v>
+        <v>152.4</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1125,11 +1135,7 @@
           <t>08-Oct-26</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1152,12 +1158,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>MINFIN / UGD</t>
+          <t>MINFIN/UGD (stated stock; the five listed bonds sum to $8.0B, unreconciled)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>30-Sep-26</t>
+          <t>Sep-26</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
@@ -1354,8 +1360,14 @@
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" t="inlineStr"/>
+      <c r="C2" s="2" t="n">
+        <v>152.4</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>IMF WEO, 08-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1369,7 +1381,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>IMF, 01-May-26</t>
+          <t>IMF, 08-Oct-26</t>
         </is>
       </c>
     </row>
@@ -1395,7 +1407,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>IMF / BNA, 01-May-26</t>
+          <t>IMF/BNA, 08-Oct-26</t>
         </is>
       </c>
     </row>
@@ -1406,8 +1418,14 @@
         </is>
       </c>
       <c r="B6" s="2" t="n"/>
-      <c r="C6" s="2" t="n"/>
-      <c r="D6" t="inlineStr"/>
+      <c r="C6" s="2" t="n">
+        <v>-2.4</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>IMF WEO, 08-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1431,7 +1449,7 @@
       <c r="C8" s="2" t="n"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>MINFIN / IMF, 01-May-26</t>
+          <t>MINFIN/IMF, May-26</t>
         </is>
       </c>
     </row>

</xml_diff>